<commit_message>
implement the email services
</commit_message>
<xml_diff>
--- a/student_template.xlsx
+++ b/student_template.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -429,7 +429,12 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Batch</t>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Year</t>
         </is>
       </c>
     </row>

</xml_diff>